<commit_message>
Edited Manual, NW design, and k8s manifest files
</commit_message>
<xml_diff>
--- a/docs/Design/NW/NW_design_byosg.xlsx
+++ b/docs/Design/NW/NW_design_byosg.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ryota/Documents/研鑽/技術/Projects/20250110_KubernetesAPI/graphapp/docs/Design/NW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC69A408-D53C-9C42-A66C-20A2E51B59A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDF20D65-6B08-6441-8EED-9221D5604F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10060" yWindow="660" windowWidth="22340" windowHeight="20180" activeTab="2" xr2:uid="{A262E15D-8A74-E342-96E0-9E111D7ACA0C}"/>
   </bookViews>
@@ -190,7 +190,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -206,6 +206,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -274,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -289,16 +301,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -315,6 +327,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10156,28 +10180,28 @@
       <c r="E2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" s="18" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>